<commit_message>
Actualización del registro de asistencias
</commit_message>
<xml_diff>
--- a/registro_asistencia/registro_estancias.xlsx
+++ b/registro_asistencia/registro_estancias.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\José Antonio\Desktop\ESTANCIAS\registro_asistencia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elisa\Desktop\ESTANCIAS_ELI\jen-estancias\registro_asistencia\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C3F7797-78DC-4FC1-9400-845E8C8F1C92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="12990" windowHeight="6300" activeTab="1"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="17940" windowHeight="9840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Jose Antonio" sheetId="2" r:id="rId1"/>
@@ -21,23 +22,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="34">
   <si>
     <t>Alumno/a:</t>
   </si>
@@ -121,12 +111,30 @@
   </si>
   <si>
     <t>4 SEMANA</t>
+  </si>
+  <si>
+    <t>Planificando la creación de videos</t>
+  </si>
+  <si>
+    <t>casa</t>
+  </si>
+  <si>
+    <t>Organización de recursos para cada video</t>
+  </si>
+  <si>
+    <t>Planificando la creación de una página web</t>
+  </si>
+  <si>
+    <t>Organización de recursos para la página web</t>
+  </si>
+  <si>
+    <t>Creación de los primeros vídeos</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="h:mm;@"/>
   </numFmts>
@@ -293,36 +301,32 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
     <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="14" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="5" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="14" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -333,23 +337,14 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="14" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -435,7 +430,6 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -455,6 +449,7 @@
           <bgColor theme="0"/>
         </patternFill>
       </fill>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -468,65 +463,6 @@
         <name val="Calibri"/>
         <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="h:mm;@"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
@@ -626,6 +562,65 @@
         <scheme val="minor"/>
       </font>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="h:mm;@"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -640,45 +635,45 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="10" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="21" dataDxfId="20" headerRowCellStyle="Énfasis1">
-  <autoFilter ref="B6:G51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="10" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Tabla811" displayName="Tabla811" ref="B6:G51" totalsRowShown="0" headerRowDxfId="14" dataDxfId="13" headerRowCellStyle="Énfasis1">
+  <autoFilter ref="B6:G51" xr:uid="{00000000-0009-0000-0100-00000A000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Fecha" dataDxfId="19"/>
-    <tableColumn id="2" name="Hora inicio" dataDxfId="18"/>
-    <tableColumn id="3" name="Hora fin" dataDxfId="17"/>
-    <tableColumn id="4" name="Tareas realizadas" dataDxfId="9"/>
-    <tableColumn id="5" name="Tiempo dedicado (h)" dataDxfId="7"/>
-    <tableColumn id="6" name="Lugar de realización" dataDxfId="8"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Fecha" dataDxfId="12"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Hora inicio" dataDxfId="11"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Hora fin" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Tareas realizadas" dataDxfId="9"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="Tiempo dedicado (h)" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="Lugar de realización" dataDxfId="7"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
-  <autoFilter ref="B6:G51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="Tabla810" displayName="Tabla810" ref="B6:G51" totalsRowShown="0" dataDxfId="21" headerRowCellStyle="Énfasis1">
+  <autoFilter ref="B6:G51" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Fecha" dataDxfId="5"/>
-    <tableColumn id="2" name="Hora inicio" dataDxfId="4"/>
-    <tableColumn id="3" name="Hora fin" dataDxfId="3"/>
-    <tableColumn id="4" name="Tareas realizadas" dataDxfId="2"/>
-    <tableColumn id="5" name="Tiempo dedicado (h)" dataDxfId="1"/>
-    <tableColumn id="6" name="Lugar de realización" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Fecha" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Hora inicio" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Hora fin" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0100-000004000000}" name="Tareas realizadas" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0100-000005000000}" name="Tiempo dedicado (h)" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0100-000006000000}" name="Lugar de realización" dataDxfId="15"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="8" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="16" headerRowCellStyle="Énfasis1">
-  <autoFilter ref="B6:G51"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="Tabla8" displayName="Tabla8" ref="B6:G51" totalsRowShown="0" dataDxfId="6" headerRowCellStyle="Énfasis1">
+  <autoFilter ref="B6:G51" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="6">
-    <tableColumn id="1" name="Fecha" dataDxfId="15"/>
-    <tableColumn id="2" name="Hora inicio" dataDxfId="14"/>
-    <tableColumn id="3" name="Hora fin" dataDxfId="13"/>
-    <tableColumn id="4" name="Tareas realizadas" dataDxfId="12"/>
-    <tableColumn id="5" name="Tiempo dedicado (h)" dataDxfId="11"/>
-    <tableColumn id="6" name="Lugar de realización" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Fecha" dataDxfId="5"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Hora inicio" dataDxfId="4"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Hora fin" dataDxfId="3"/>
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0200-000004000000}" name="Tareas realizadas" dataDxfId="2"/>
+    <tableColumn id="5" xr3:uid="{00000000-0010-0000-0200-000005000000}" name="Tiempo dedicado (h)" dataDxfId="1"/>
+    <tableColumn id="6" xr3:uid="{00000000-0010-0000-0200-000006000000}" name="Lugar de realización" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium23" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -968,7 +963,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -985,65 +980,65 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="20"/>
+      <c r="D2" s="24"/>
+      <c r="E2" s="24"/>
+      <c r="F2" s="24"/>
+      <c r="G2" s="25"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="15"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
+      <c r="B3" s="11"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="20"/>
+      <c r="D4" s="24"/>
+      <c r="E4" s="24"/>
+      <c r="F4" s="24"/>
+      <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
       <c r="N5" s="5" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="3" t="s">
         <v>8</v>
       </c>
       <c r="N6" s="5" t="s">
@@ -1051,25 +1046,25 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B7" s="13">
         <v>46118</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="17">
         <v>6</v>
       </c>
-      <c r="G7" s="30" t="s">
+      <c r="G7" s="16" t="s">
         <v>2</v>
       </c>
       <c r="N7" s="5" t="s">
@@ -1077,556 +1072,586 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="27">
+      <c r="A8" s="19"/>
+      <c r="B8" s="13">
         <v>46118</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="15">
         <v>0.75</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="17">
         <v>2</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="G8" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="34"/>
-      <c r="B9" s="27">
+      <c r="A9" s="19"/>
+      <c r="B9" s="13">
         <v>46119</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="14">
         <v>0.39583333333333331</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="15">
         <v>0.5625</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="17">
         <v>4</v>
       </c>
-      <c r="G9" s="30" t="s">
+      <c r="G9" s="16" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="27">
+      <c r="A10" s="19"/>
+      <c r="B10" s="13">
         <v>46119</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="15">
         <v>0.83333333333333337</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="17">
         <v>4</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="27">
+      <c r="A11" s="19"/>
+      <c r="B11" s="13">
         <v>46120</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="31">
+      <c r="F11" s="17">
         <v>6</v>
       </c>
-      <c r="G11" s="30" t="s">
+      <c r="G11" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="27">
+      <c r="A12" s="19"/>
+      <c r="B12" s="13">
         <v>46120</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="15">
         <v>0.75</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="17">
         <v>2</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="27">
+      <c r="A13" s="19"/>
+      <c r="B13" s="13">
         <v>46121</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="17">
         <v>6</v>
       </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="27">
+      <c r="A14" s="19"/>
+      <c r="B14" s="13">
         <v>46121</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="15">
         <v>0.64583333333333337</v>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="15">
         <v>0.72916666666666663</v>
       </c>
-      <c r="E14" s="33" t="s">
+      <c r="E14" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="17">
         <v>2</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
-      <c r="B15" s="27">
+      <c r="A15" s="19"/>
+      <c r="B15" s="13">
         <v>46122</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="15">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E15" s="33" t="s">
+      <c r="E15" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="17">
         <v>6</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="27">
+      <c r="A16" s="19"/>
+      <c r="B16" s="13">
         <v>46122</v>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="15">
         <v>0.75</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="17">
         <v>2</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="7">
         <v>46125</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="E17" s="1"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="1"/>
+      <c r="C17" s="4">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="F17" s="12">
+        <v>6</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="11">
+      <c r="A18" s="19"/>
+      <c r="B18" s="7">
         <v>46125</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="E18" s="1"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="1"/>
+      <c r="C18" s="4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F18" s="12">
+        <v>2</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="11">
+      <c r="A19" s="19"/>
+      <c r="B19" s="7">
         <v>46126</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="E19" s="1"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="1"/>
+      <c r="C19" s="4">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="12">
+        <v>6</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="34"/>
-      <c r="B20" s="11">
+      <c r="A20" s="19"/>
+      <c r="B20" s="7">
         <v>46126</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
       <c r="E20" s="1"/>
-      <c r="F20" s="25"/>
+      <c r="F20" s="12"/>
       <c r="G20" s="1"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="34"/>
-      <c r="B21" s="11">
+      <c r="A21" s="19"/>
+      <c r="B21" s="7">
         <v>46127</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
       <c r="E21" s="1"/>
-      <c r="F21" s="25"/>
+      <c r="F21" s="12"/>
       <c r="G21" s="1"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="34"/>
-      <c r="B22" s="11">
+      <c r="A22" s="19"/>
+      <c r="B22" s="7">
         <v>46127</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
       <c r="E22" s="1"/>
-      <c r="F22" s="25"/>
+      <c r="F22" s="12"/>
       <c r="G22" s="1"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="34"/>
-      <c r="B23" s="11">
+      <c r="A23" s="19"/>
+      <c r="B23" s="7">
         <v>46128</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
       <c r="E23" s="1"/>
-      <c r="F23" s="25"/>
+      <c r="F23" s="12"/>
       <c r="G23" s="1"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="34"/>
-      <c r="B24" s="11">
+      <c r="A24" s="19"/>
+      <c r="B24" s="7">
         <v>46128</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
       <c r="E24" s="1"/>
-      <c r="F24" s="25"/>
+      <c r="F24" s="12"/>
       <c r="G24" s="1"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="34"/>
-      <c r="B25" s="11">
+      <c r="A25" s="19"/>
+      <c r="B25" s="7">
         <v>46129</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
       <c r="E25" s="1"/>
-      <c r="F25" s="25"/>
+      <c r="F25" s="12"/>
       <c r="G25" s="1"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="34"/>
-      <c r="B26" s="11">
+      <c r="A26" s="19"/>
+      <c r="B26" s="7">
         <v>46129</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
       <c r="E26" s="1"/>
-      <c r="F26" s="25"/>
+      <c r="F26" s="12"/>
       <c r="G26" s="1"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="13">
         <v>46132</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="33"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="34"/>
-      <c r="B28" s="27">
+      <c r="A28" s="19"/>
+      <c r="B28" s="13">
         <v>46132</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="33"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="34"/>
-      <c r="B29" s="27">
+      <c r="A29" s="19"/>
+      <c r="B29" s="13">
         <v>46133</v>
       </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="33"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="34"/>
-      <c r="B30" s="27">
+      <c r="A30" s="19"/>
+      <c r="B30" s="13">
         <v>46133</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="33"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="34"/>
-      <c r="B31" s="27">
+      <c r="A31" s="19"/>
+      <c r="B31" s="13">
         <v>46134</v>
       </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="33"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="34"/>
-      <c r="B32" s="27">
+      <c r="A32" s="19"/>
+      <c r="B32" s="13">
         <v>46134</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="33"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="34"/>
-      <c r="B33" s="27">
+      <c r="A33" s="19"/>
+      <c r="B33" s="13">
         <v>46135</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="33"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="34"/>
-      <c r="B34" s="27">
+      <c r="A34" s="19"/>
+      <c r="B34" s="13">
         <v>46135</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="33"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
-      <c r="B35" s="27">
+      <c r="A35" s="19"/>
+      <c r="B35" s="13">
         <v>46136</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="33"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="34"/>
-      <c r="B36" s="27">
+      <c r="A36" s="19"/>
+      <c r="B36" s="13">
         <v>46136</v>
       </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="33"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="34" t="s">
+      <c r="A37" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="7">
         <v>46139</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
       <c r="E37" s="1"/>
-      <c r="F37" s="25"/>
+      <c r="F37" s="12"/>
       <c r="G37" s="1"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B38" s="11">
+      <c r="B38" s="7">
         <v>46139</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
       <c r="E38" s="1"/>
-      <c r="F38" s="25"/>
+      <c r="F38" s="12"/>
       <c r="G38" s="1"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B39" s="11">
+      <c r="B39" s="7">
         <v>46140</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
       <c r="E39" s="1"/>
-      <c r="F39" s="25"/>
+      <c r="F39" s="12"/>
       <c r="G39" s="1"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B40" s="11">
+      <c r="B40" s="7">
         <v>46140</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
       <c r="E40" s="1"/>
-      <c r="F40" s="25"/>
+      <c r="F40" s="12"/>
       <c r="G40" s="1"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B41" s="11">
+      <c r="B41" s="7">
         <v>46141</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
       <c r="E41" s="1"/>
-      <c r="F41" s="25"/>
+      <c r="F41" s="12"/>
       <c r="G41" s="1"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B42" s="11">
+      <c r="B42" s="7">
         <v>46141</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
       <c r="E42" s="1"/>
-      <c r="F42" s="25"/>
+      <c r="F42" s="12"/>
       <c r="G42" s="1"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B43" s="11">
+      <c r="B43" s="7">
         <v>46142</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
       <c r="E43" s="1"/>
-      <c r="F43" s="25"/>
+      <c r="F43" s="12"/>
       <c r="G43" s="1"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B44" s="11">
+      <c r="B44" s="7">
         <v>46142</v>
       </c>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="9"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="E44" s="1"/>
+      <c r="F44" s="12"/>
+      <c r="G44" s="1"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B45" s="6"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="9"/>
-      <c r="F45" s="26"/>
-      <c r="G45" s="9"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="4"/>
+      <c r="D45" s="4"/>
+      <c r="E45" s="1"/>
+      <c r="F45" s="12"/>
+      <c r="G45" s="1"/>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B46" s="6"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="26"/>
-      <c r="G46" s="9"/>
+      <c r="B46" s="2"/>
+      <c r="C46" s="4"/>
+      <c r="D46" s="4"/>
+      <c r="E46" s="1"/>
+      <c r="F46" s="12"/>
+      <c r="G46" s="1"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B47" s="6"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="9"/>
-      <c r="F47" s="26"/>
-      <c r="G47" s="9"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="4"/>
+      <c r="D47" s="4"/>
+      <c r="E47" s="1"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="1"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B48" s="6"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="9"/>
-      <c r="F48" s="26"/>
-      <c r="G48" s="9"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="4"/>
+      <c r="D48" s="4"/>
+      <c r="E48" s="1"/>
+      <c r="F48" s="12"/>
+      <c r="G48" s="1"/>
     </row>
     <row r="49" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B49" s="6"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="9"/>
-      <c r="F49" s="26"/>
-      <c r="G49" s="9"/>
+      <c r="B49" s="2"/>
+      <c r="C49" s="4"/>
+      <c r="D49" s="4"/>
+      <c r="E49" s="1"/>
+      <c r="F49" s="12"/>
+      <c r="G49" s="1"/>
     </row>
     <row r="50" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B50" s="6"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="9"/>
-      <c r="F50" s="26"/>
-      <c r="G50" s="9"/>
+      <c r="B50" s="2"/>
+      <c r="C50" s="4"/>
+      <c r="D50" s="4"/>
+      <c r="E50" s="1"/>
+      <c r="F50" s="12"/>
+      <c r="G50" s="1"/>
     </row>
     <row r="51" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B51" s="6"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="9"/>
-      <c r="F51" s="26"/>
-      <c r="G51" s="9"/>
+      <c r="B51" s="2"/>
+      <c r="C51" s="4"/>
+      <c r="D51" s="4"/>
+      <c r="E51" s="1"/>
+      <c r="F51" s="12"/>
+      <c r="G51" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -1634,7 +1659,7 @@
     <mergeCell ref="C4:G4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G35:G51 G7 G9 G11 G13 G15 G17 G19 G21 G23 G25 G27 G29 G31 G33">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G35:G51 G7 G9 G11 G13 G15 G33 G19 G21 G23 G25 G27 G29 G31 G17" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$N$5:$N$7</formula1>
     </dataValidation>
   </dataValidations>
@@ -1647,7 +1672,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1664,31 +1689,31 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="20" t="s">
         <v>15</v>
       </c>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="24"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="17"/>
+      <c r="B3" s="11"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="24"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -1719,25 +1744,25 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B7" s="13">
         <v>46118</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="17">
         <v>6</v>
       </c>
-      <c r="G7" s="30" t="s">
+      <c r="G7" s="16" t="s">
         <v>2</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -1745,473 +1770,507 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="27">
+      <c r="A8" s="19"/>
+      <c r="B8" s="13">
         <v>46118</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="15">
         <v>0.75</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="17">
         <v>2</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="G8" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="34"/>
-      <c r="B9" s="27">
+      <c r="A9" s="19"/>
+      <c r="B9" s="13">
         <v>46119</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="14">
         <v>0.39583333333333331</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="15">
         <v>0.5625</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="17">
         <v>4</v>
       </c>
-      <c r="G9" s="30" t="s">
+      <c r="G9" s="16" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="27">
+      <c r="A10" s="19"/>
+      <c r="B10" s="13">
         <v>46119</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="15">
         <v>0.83333333333333337</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="17">
         <v>4</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="27">
+      <c r="A11" s="19"/>
+      <c r="B11" s="13">
         <v>46120</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="31">
+      <c r="F11" s="17">
         <v>6</v>
       </c>
-      <c r="G11" s="30" t="s">
+      <c r="G11" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="27">
+      <c r="A12" s="19"/>
+      <c r="B12" s="13">
         <v>46120</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="15">
         <v>0.75</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="17">
         <v>2</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="27">
+      <c r="A13" s="19"/>
+      <c r="B13" s="13">
         <v>46121</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="17">
         <v>6</v>
       </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="27">
+      <c r="A14" s="19"/>
+      <c r="B14" s="13">
         <v>46121</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="15">
         <v>0.64583333333333337</v>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="15">
         <v>0.72916666666666663</v>
       </c>
-      <c r="E14" s="33" t="s">
+      <c r="E14" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="17">
         <v>2</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
-      <c r="B15" s="27">
+      <c r="A15" s="19"/>
+      <c r="B15" s="13">
         <v>46122</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="15">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E15" s="33" t="s">
+      <c r="E15" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="17">
         <v>6</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="27">
+      <c r="A16" s="19"/>
+      <c r="B16" s="13">
         <v>46122</v>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="15">
         <v>0.75</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="17">
         <v>2</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="7">
         <v>46125</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="F17" s="25"/>
+      <c r="C17" s="4">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="12">
+        <v>6</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="11">
+      <c r="A18" s="19"/>
+      <c r="B18" s="7">
         <v>46125</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="F18" s="25"/>
+      <c r="C18" s="4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="12">
+        <v>2</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="11">
+      <c r="A19" s="19"/>
+      <c r="B19" s="7">
         <v>46126</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="F19" s="25"/>
+      <c r="C19" s="4">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="12">
+        <v>6</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="34"/>
-      <c r="B20" s="11">
+      <c r="A20" s="19"/>
+      <c r="B20" s="7">
         <v>46126</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
-      <c r="F20" s="25"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="34"/>
-      <c r="B21" s="11">
+      <c r="A21" s="19"/>
+      <c r="B21" s="7">
         <v>46127</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="F21" s="25"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="34"/>
-      <c r="B22" s="11">
+      <c r="A22" s="19"/>
+      <c r="B22" s="7">
         <v>46127</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="F22" s="25"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="34"/>
-      <c r="B23" s="11">
+      <c r="A23" s="19"/>
+      <c r="B23" s="7">
         <v>46128</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="F23" s="25"/>
+      <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="34"/>
-      <c r="B24" s="11">
+      <c r="A24" s="19"/>
+      <c r="B24" s="7">
         <v>46128</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="F24" s="25"/>
+      <c r="F24" s="12"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="34"/>
-      <c r="B25" s="11">
+      <c r="A25" s="19"/>
+      <c r="B25" s="7">
         <v>46129</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="F25" s="25"/>
+      <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="34"/>
-      <c r="B26" s="11">
+      <c r="A26" s="19"/>
+      <c r="B26" s="7">
         <v>46129</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
-      <c r="F26" s="25"/>
+      <c r="F26" s="12"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="13">
         <v>46132</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="33"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="34"/>
-      <c r="B28" s="27">
+      <c r="A28" s="19"/>
+      <c r="B28" s="13">
         <v>46132</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="33"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="34"/>
-      <c r="B29" s="27">
+      <c r="A29" s="19"/>
+      <c r="B29" s="13">
         <v>46133</v>
       </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="33"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="34"/>
-      <c r="B30" s="27">
+      <c r="A30" s="19"/>
+      <c r="B30" s="13">
         <v>46133</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="33"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="34"/>
-      <c r="B31" s="27">
+      <c r="A31" s="19"/>
+      <c r="B31" s="13">
         <v>46134</v>
       </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="33"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="34"/>
-      <c r="B32" s="27">
+      <c r="A32" s="19"/>
+      <c r="B32" s="13">
         <v>46134</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="33"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="34"/>
-      <c r="B33" s="27">
+      <c r="A33" s="19"/>
+      <c r="B33" s="13">
         <v>46135</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="33"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="34"/>
-      <c r="B34" s="27">
+      <c r="A34" s="19"/>
+      <c r="B34" s="13">
         <v>46135</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="33"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
-      <c r="B35" s="27">
+      <c r="A35" s="19"/>
+      <c r="B35" s="13">
         <v>46136</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="33"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="34"/>
-      <c r="B36" s="27">
+      <c r="A36" s="19"/>
+      <c r="B36" s="13">
         <v>46136</v>
       </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="33"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="34" t="s">
+      <c r="A37" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="7">
         <v>46139</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="F37" s="25"/>
+      <c r="F37" s="12"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
-      <c r="B38" s="11">
+      <c r="B38" s="7">
         <v>46139</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="F38" s="25"/>
+      <c r="F38" s="12"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
-      <c r="B39" s="11">
+      <c r="B39" s="7">
         <v>46140</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="F39" s="25"/>
+      <c r="F39" s="12"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
-      <c r="B40" s="11">
+      <c r="B40" s="7">
         <v>46140</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="F40" s="25"/>
+      <c r="F40" s="12"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
-      <c r="B41" s="11">
+      <c r="B41" s="7">
         <v>46141</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="F41" s="25"/>
+      <c r="F41" s="12"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
-      <c r="B42" s="11">
+      <c r="B42" s="7">
         <v>46141</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="F42" s="25"/>
+      <c r="F42" s="12"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
-      <c r="B43" s="11">
+      <c r="B43" s="7">
         <v>46142</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="F43" s="25"/>
+      <c r="F43" s="12"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
-      <c r="B44" s="11">
+      <c r="B44" s="7">
         <v>46142</v>
       </c>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="9"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="F44" s="12"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
@@ -2254,7 +2313,7 @@
     <mergeCell ref="C4:G4"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G35:G51 G7 G9 G11 G13 G15 G17 G19 G21 G23 G25 G27 G29 G31 G33">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G35:G51 G7 G9 G11 G13 G15 G17 G33 G21 G23 G25 G27 G29 G31 G19" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>$N$5:$N$7</formula1>
     </dataValidation>
   </dataValidations>
@@ -2266,7 +2325,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:N51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -2283,32 +2342,32 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="C2" s="20" t="s">
         <v>16</v>
       </c>
-      <c r="D2" s="23"/>
-      <c r="E2" s="23"/>
-      <c r="F2" s="23"/>
-      <c r="G2" s="24"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="22"/>
     </row>
     <row r="3" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="14"/>
-      <c r="C3" s="13"/>
+      <c r="B3" s="10"/>
+      <c r="C3" s="9"/>
     </row>
     <row r="4" spans="1:14" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="12" t="s">
+      <c r="B4" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="22" t="s">
+      <c r="C4" s="20" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="23"/>
-      <c r="E4" s="23"/>
-      <c r="F4" s="23"/>
-      <c r="G4" s="24"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="22"/>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N5" s="1" t="s">
@@ -2339,25 +2398,25 @@
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" s="34" t="s">
+      <c r="A7" s="19" t="s">
         <v>25</v>
       </c>
-      <c r="B7" s="27">
+      <c r="B7" s="13">
         <v>46118</v>
       </c>
-      <c r="C7" s="28">
+      <c r="C7" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D7" s="29">
+      <c r="D7" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E7" s="30" t="s">
+      <c r="E7" s="16" t="s">
         <v>12</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="17">
         <v>6</v>
       </c>
-      <c r="G7" s="30" t="s">
+      <c r="G7" s="16" t="s">
         <v>2</v>
       </c>
       <c r="N7" s="1" t="s">
@@ -2365,473 +2424,507 @@
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="34"/>
-      <c r="B8" s="27">
+      <c r="A8" s="19"/>
+      <c r="B8" s="13">
         <v>46118</v>
       </c>
-      <c r="C8" s="29">
+      <c r="C8" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D8" s="29">
+      <c r="D8" s="15">
         <v>0.75</v>
       </c>
-      <c r="E8" s="32" t="s">
+      <c r="E8" s="18" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="31">
+      <c r="F8" s="17">
         <v>2</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="G8" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" s="34"/>
-      <c r="B9" s="27">
+      <c r="A9" s="19"/>
+      <c r="B9" s="13">
         <v>46119</v>
       </c>
-      <c r="C9" s="28">
+      <c r="C9" s="14">
         <v>0.39583333333333331</v>
       </c>
-      <c r="D9" s="29">
+      <c r="D9" s="15">
         <v>0.5625</v>
       </c>
-      <c r="E9" s="30" t="s">
+      <c r="E9" s="16" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="17">
         <v>4</v>
       </c>
-      <c r="G9" s="30" t="s">
+      <c r="G9" s="16" t="s">
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" s="34"/>
-      <c r="B10" s="27">
+      <c r="A10" s="19"/>
+      <c r="B10" s="13">
         <v>46119</v>
       </c>
-      <c r="C10" s="29">
+      <c r="C10" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D10" s="29">
+      <c r="D10" s="15">
         <v>0.83333333333333337</v>
       </c>
-      <c r="E10" s="33" t="s">
+      <c r="E10" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="F10" s="31">
+      <c r="F10" s="17">
         <v>4</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" s="34"/>
-      <c r="B11" s="27">
+      <c r="A11" s="19"/>
+      <c r="B11" s="13">
         <v>46120</v>
       </c>
-      <c r="C11" s="28">
+      <c r="C11" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D11" s="29">
+      <c r="D11" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E11" s="32" t="s">
+      <c r="E11" s="18" t="s">
         <v>19</v>
       </c>
-      <c r="F11" s="31">
+      <c r="F11" s="17">
         <v>6</v>
       </c>
-      <c r="G11" s="30" t="s">
+      <c r="G11" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A12" s="34"/>
-      <c r="B12" s="27">
+      <c r="A12" s="19"/>
+      <c r="B12" s="13">
         <v>46120</v>
       </c>
-      <c r="C12" s="29">
+      <c r="C12" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D12" s="29">
+      <c r="D12" s="15">
         <v>0.75</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="E12" s="18" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="31">
+      <c r="F12" s="17">
         <v>2</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A13" s="34"/>
-      <c r="B13" s="27">
+      <c r="A13" s="19"/>
+      <c r="B13" s="13">
         <v>46121</v>
       </c>
-      <c r="C13" s="28">
+      <c r="C13" s="14">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D13" s="29">
+      <c r="D13" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E13" s="33" t="s">
+      <c r="E13" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="31">
+      <c r="F13" s="17">
         <v>6</v>
       </c>
-      <c r="G13" s="30" t="s">
+      <c r="G13" s="16" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A14" s="34"/>
-      <c r="B14" s="27">
+      <c r="A14" s="19"/>
+      <c r="B14" s="13">
         <v>46121</v>
       </c>
-      <c r="C14" s="29">
+      <c r="C14" s="15">
         <v>0.64583333333333337</v>
       </c>
-      <c r="D14" s="29">
+      <c r="D14" s="15">
         <v>0.72916666666666663</v>
       </c>
-      <c r="E14" s="33" t="s">
+      <c r="E14" s="18" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="31">
+      <c r="F14" s="17">
         <v>2</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A15" s="34"/>
-      <c r="B15" s="27">
+      <c r="A15" s="19"/>
+      <c r="B15" s="13">
         <v>46122</v>
       </c>
-      <c r="C15" s="29">
+      <c r="C15" s="15">
         <v>0.35416666666666669</v>
       </c>
-      <c r="D15" s="29">
+      <c r="D15" s="15">
         <v>0.60416666666666663</v>
       </c>
-      <c r="E15" s="33" t="s">
+      <c r="E15" s="18" t="s">
         <v>22</v>
       </c>
-      <c r="F15" s="31">
+      <c r="F15" s="17">
         <v>6</v>
       </c>
-      <c r="G15" s="33" t="s">
+      <c r="G15" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A16" s="34"/>
-      <c r="B16" s="27">
+      <c r="A16" s="19"/>
+      <c r="B16" s="13">
         <v>46122</v>
       </c>
-      <c r="C16" s="29">
+      <c r="C16" s="15">
         <v>0.66666666666666663</v>
       </c>
-      <c r="D16" s="29">
+      <c r="D16" s="15">
         <v>0.75</v>
       </c>
-      <c r="E16" s="33" t="s">
+      <c r="E16" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="31">
+      <c r="F16" s="17">
         <v>2</v>
       </c>
-      <c r="G16" s="33" t="s">
+      <c r="G16" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="34" t="s">
+      <c r="A17" s="19" t="s">
         <v>24</v>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="7">
         <v>46125</v>
       </c>
-      <c r="C17" s="4"/>
-      <c r="D17" s="4"/>
-      <c r="F17" s="25"/>
+      <c r="C17" s="4">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D17" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="12">
+        <v>6</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="34"/>
-      <c r="B18" s="11">
+      <c r="A18" s="19"/>
+      <c r="B18" s="7">
         <v>46125</v>
       </c>
-      <c r="C18" s="4"/>
-      <c r="D18" s="4"/>
-      <c r="F18" s="25"/>
+      <c r="C18" s="4">
+        <v>0.66666666666666663</v>
+      </c>
+      <c r="D18" s="4">
+        <v>0.75</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F18" s="12">
+        <v>2</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="34"/>
-      <c r="B19" s="11">
+      <c r="A19" s="19"/>
+      <c r="B19" s="7">
         <v>46126</v>
       </c>
-      <c r="C19" s="4"/>
-      <c r="D19" s="4"/>
-      <c r="F19" s="25"/>
+      <c r="C19" s="4">
+        <v>0.35416666666666669</v>
+      </c>
+      <c r="D19" s="4">
+        <v>0.60416666666666663</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F19" s="12">
+        <v>6</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>2</v>
+      </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="34"/>
-      <c r="B20" s="11">
+      <c r="A20" s="19"/>
+      <c r="B20" s="7">
         <v>46126</v>
       </c>
       <c r="C20" s="4"/>
       <c r="D20" s="4"/>
-      <c r="F20" s="25"/>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="34"/>
-      <c r="B21" s="11">
+      <c r="A21" s="19"/>
+      <c r="B21" s="7">
         <v>46127</v>
       </c>
       <c r="C21" s="4"/>
       <c r="D21" s="4"/>
-      <c r="F21" s="25"/>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="34"/>
-      <c r="B22" s="11">
+      <c r="A22" s="19"/>
+      <c r="B22" s="7">
         <v>46127</v>
       </c>
       <c r="C22" s="4"/>
       <c r="D22" s="4"/>
-      <c r="F22" s="25"/>
+      <c r="F22" s="12"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="34"/>
-      <c r="B23" s="11">
+      <c r="A23" s="19"/>
+      <c r="B23" s="7">
         <v>46128</v>
       </c>
       <c r="C23" s="4"/>
       <c r="D23" s="4"/>
-      <c r="F23" s="25"/>
+      <c r="F23" s="12"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="34"/>
-      <c r="B24" s="11">
+      <c r="A24" s="19"/>
+      <c r="B24" s="7">
         <v>46128</v>
       </c>
       <c r="C24" s="4"/>
       <c r="D24" s="4"/>
-      <c r="F24" s="25"/>
+      <c r="F24" s="12"/>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="34"/>
-      <c r="B25" s="11">
+      <c r="A25" s="19"/>
+      <c r="B25" s="7">
         <v>46129</v>
       </c>
       <c r="C25" s="4"/>
       <c r="D25" s="4"/>
-      <c r="F25" s="25"/>
+      <c r="F25" s="12"/>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="34"/>
-      <c r="B26" s="11">
+      <c r="A26" s="19"/>
+      <c r="B26" s="7">
         <v>46129</v>
       </c>
       <c r="C26" s="4"/>
       <c r="D26" s="4"/>
-      <c r="F26" s="25"/>
+      <c r="F26" s="12"/>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="34" t="s">
+      <c r="A27" s="19" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="27">
+      <c r="B27" s="13">
         <v>46132</v>
       </c>
-      <c r="C27" s="29"/>
-      <c r="D27" s="29"/>
-      <c r="E27" s="33"/>
-      <c r="F27" s="31"/>
-      <c r="G27" s="33"/>
+      <c r="C27" s="15"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="18"/>
+      <c r="F27" s="17"/>
+      <c r="G27" s="18"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="34"/>
-      <c r="B28" s="27">
+      <c r="A28" s="19"/>
+      <c r="B28" s="13">
         <v>46132</v>
       </c>
-      <c r="C28" s="29"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="31"/>
-      <c r="G28" s="33"/>
+      <c r="C28" s="15"/>
+      <c r="D28" s="15"/>
+      <c r="E28" s="18"/>
+      <c r="F28" s="17"/>
+      <c r="G28" s="18"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="34"/>
-      <c r="B29" s="27">
+      <c r="A29" s="19"/>
+      <c r="B29" s="13">
         <v>46133</v>
       </c>
-      <c r="C29" s="29"/>
-      <c r="D29" s="29"/>
-      <c r="E29" s="33"/>
-      <c r="F29" s="31"/>
-      <c r="G29" s="33"/>
+      <c r="C29" s="15"/>
+      <c r="D29" s="15"/>
+      <c r="E29" s="18"/>
+      <c r="F29" s="17"/>
+      <c r="G29" s="18"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="34"/>
-      <c r="B30" s="27">
+      <c r="A30" s="19"/>
+      <c r="B30" s="13">
         <v>46133</v>
       </c>
-      <c r="C30" s="29"/>
-      <c r="D30" s="29"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="31"/>
-      <c r="G30" s="33"/>
+      <c r="C30" s="15"/>
+      <c r="D30" s="15"/>
+      <c r="E30" s="18"/>
+      <c r="F30" s="17"/>
+      <c r="G30" s="18"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="34"/>
-      <c r="B31" s="27">
+      <c r="A31" s="19"/>
+      <c r="B31" s="13">
         <v>46134</v>
       </c>
-      <c r="C31" s="29"/>
-      <c r="D31" s="29"/>
-      <c r="E31" s="33"/>
-      <c r="F31" s="31"/>
-      <c r="G31" s="33"/>
+      <c r="C31" s="15"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="18"/>
+      <c r="F31" s="17"/>
+      <c r="G31" s="18"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="34"/>
-      <c r="B32" s="27">
+      <c r="A32" s="19"/>
+      <c r="B32" s="13">
         <v>46134</v>
       </c>
-      <c r="C32" s="29"/>
-      <c r="D32" s="29"/>
-      <c r="E32" s="33"/>
-      <c r="F32" s="31"/>
-      <c r="G32" s="33"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="18"/>
+      <c r="F32" s="17"/>
+      <c r="G32" s="18"/>
     </row>
     <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" s="34"/>
-      <c r="B33" s="27">
+      <c r="A33" s="19"/>
+      <c r="B33" s="13">
         <v>46135</v>
       </c>
-      <c r="C33" s="29"/>
-      <c r="D33" s="29"/>
-      <c r="E33" s="33"/>
-      <c r="F33" s="31"/>
-      <c r="G33" s="33"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="18"/>
+      <c r="F33" s="17"/>
+      <c r="G33" s="18"/>
     </row>
     <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" s="34"/>
-      <c r="B34" s="27">
+      <c r="A34" s="19"/>
+      <c r="B34" s="13">
         <v>46135</v>
       </c>
-      <c r="C34" s="29"/>
-      <c r="D34" s="29"/>
-      <c r="E34" s="33"/>
-      <c r="F34" s="31"/>
-      <c r="G34" s="33"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="18"/>
+      <c r="F34" s="17"/>
+      <c r="G34" s="18"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="34"/>
-      <c r="B35" s="27">
+      <c r="A35" s="19"/>
+      <c r="B35" s="13">
         <v>46136</v>
       </c>
-      <c r="C35" s="29"/>
-      <c r="D35" s="29"/>
-      <c r="E35" s="33"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="33"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="18"/>
+      <c r="F35" s="17"/>
+      <c r="G35" s="18"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="34"/>
-      <c r="B36" s="27">
+      <c r="A36" s="19"/>
+      <c r="B36" s="13">
         <v>46136</v>
       </c>
-      <c r="C36" s="29"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="33"/>
-      <c r="F36" s="31"/>
-      <c r="G36" s="33"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="17"/>
+      <c r="G36" s="18"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="34" t="s">
+      <c r="A37" s="19" t="s">
         <v>27</v>
       </c>
-      <c r="B37" s="11">
+      <c r="B37" s="7">
         <v>46139</v>
       </c>
       <c r="C37" s="4"/>
       <c r="D37" s="4"/>
-      <c r="F37" s="25"/>
+      <c r="F37" s="12"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="5"/>
-      <c r="B38" s="11">
+      <c r="B38" s="7">
         <v>46139</v>
       </c>
       <c r="C38" s="4"/>
       <c r="D38" s="4"/>
-      <c r="F38" s="25"/>
+      <c r="F38" s="12"/>
     </row>
     <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="5"/>
-      <c r="B39" s="11">
+      <c r="B39" s="7">
         <v>46140</v>
       </c>
       <c r="C39" s="4"/>
       <c r="D39" s="4"/>
-      <c r="F39" s="25"/>
+      <c r="F39" s="12"/>
     </row>
     <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="5"/>
-      <c r="B40" s="11">
+      <c r="B40" s="7">
         <v>46140</v>
       </c>
       <c r="C40" s="4"/>
       <c r="D40" s="4"/>
-      <c r="F40" s="25"/>
+      <c r="F40" s="12"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="5"/>
-      <c r="B41" s="11">
+      <c r="B41" s="7">
         <v>46141</v>
       </c>
       <c r="C41" s="4"/>
       <c r="D41" s="4"/>
-      <c r="F41" s="25"/>
+      <c r="F41" s="12"/>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="5"/>
-      <c r="B42" s="11">
+      <c r="B42" s="7">
         <v>46141</v>
       </c>
       <c r="C42" s="4"/>
       <c r="D42" s="4"/>
-      <c r="F42" s="25"/>
+      <c r="F42" s="12"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="5"/>
-      <c r="B43" s="11">
+      <c r="B43" s="7">
         <v>46142</v>
       </c>
       <c r="C43" s="4"/>
       <c r="D43" s="4"/>
-      <c r="F43" s="25"/>
+      <c r="F43" s="12"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="5"/>
-      <c r="B44" s="11">
+      <c r="B44" s="7">
         <v>46142</v>
       </c>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="9"/>
-      <c r="F44" s="26"/>
-      <c r="G44" s="9"/>
+      <c r="C44" s="4"/>
+      <c r="D44" s="4"/>
+      <c r="F44" s="12"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="B45" s="2"/>
@@ -2874,7 +2967,7 @@
     <mergeCell ref="C2:G2"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G35:G51 G7 G9 G11 G13 G15 G17 G19 G21 G23 G25 G27 G29 G31 G33">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="G35:G51 G7 G9 G11 G13 G15 G33 G17 G21 G23 G25 G27 G29 G31 G19" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>$N$5:$N$7</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>